<commit_message>
Added dashboard test cases and updated existing validation logic
</commit_message>
<xml_diff>
--- a/Selenium_Automation/OrangeHRM-Automation/src/test/resources/DataRepository/DataRepository.xlsx
+++ b/Selenium_Automation/OrangeHRM-Automation/src/test/resources/DataRepository/DataRepository.xlsx
@@ -3,15 +3,20 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{735D4700-C3DB-45A7-BED2-9EE30BFAE69D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MyWorkspace\Selenium\OrangeHRM-Automation\src\test\resources\DataRepository\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0DF2270-C2F0-4A05-AA5C-398AF090E770}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
+    <sheet name="LoginSanity" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -21,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="30">
   <si>
     <t>Scenario Name</t>
   </si>
@@ -175,6 +180,21 @@
     <tableColumn id="4" xr3:uid="{F2690F25-322D-4432-8686-E0125242F2CB}" name="Expected Result"/>
     <tableColumn id="5" xr3:uid="{3C6AC8B4-63F7-41CF-8360-DDFC3659ADAE}" name="Priority"/>
     <tableColumn id="6" xr3:uid="{E76E6D09-5D94-4DBF-917D-095F2D1DE40F}" name="Status"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{CA71CCC3-1A3D-4721-84E4-0A6FCD6F0F28}" name="Table5" displayName="Table5" ref="A1:F2" totalsRowShown="0">
+  <autoFilter ref="A1:F2" xr:uid="{CA71CCC3-1A3D-4721-84E4-0A6FCD6F0F28}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{4171D659-142A-4F30-AF09-DFC7B22B9C2F}" name="Scenario Name"/>
+    <tableColumn id="2" xr3:uid="{36363A90-645C-4AD5-B1DB-4CA395E97ADD}" name="Username"/>
+    <tableColumn id="3" xr3:uid="{AD435456-8533-4A22-B3D7-ED8D63A4F461}" name="Password"/>
+    <tableColumn id="4" xr3:uid="{A7577607-8CC7-47EB-AECD-4DFDBC31308F}" name="Expected Result"/>
+    <tableColumn id="5" xr3:uid="{8D13790E-B931-48B0-BF51-9158A92B362C}" name="Priority"/>
+    <tableColumn id="6" xr3:uid="{F7117C7C-AB09-471F-BA60-1E73F733F3E3}" name="Status"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -593,4 +613,60 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FBE2852-F2D9-4CDC-B83A-70B3BB203037}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="6" width="10.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>